<commit_message>
docs: demonstrate missing collection recovery
</commit_message>
<xml_diff>
--- a/samples/missing_output_policies_output.xlsx
+++ b/samples/missing_output_policies_output.xlsx
@@ -533,12 +533,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -548,16 +549,18 @@
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
-      <c r="C1" s="3" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="3" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Strict mode rejects absent output values; blank and preserve modes publish warnings.</t>
+          <t>Strict mode rejects unavailable values; blank and preserve modes publish warnings.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" s="3" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -657,10 +660,103 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Null collection aggregate</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>{{ null_rows | sum }}</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Exact tag remains visible in preserve mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Missing table repeat</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>{% for row in tables["some_table"] %}{{ row.name }}</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Static body</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>{{ row.amount }}</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>{% endfor %}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Between blocks</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Unaffected</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Null collection repeat</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>{% for row in null_rows %}{{ row.name }}</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Static body</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>{{ row.amount }}</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>{% endfor %}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="C16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>